<commit_message>
Direct Write Excel for WELDING_ALUMINUM-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_WELDING_ALUMINUM-01.xlsx
+++ b/FM-MN-07_WELDING_ALUMINUM-01.xlsx
@@ -1717,7 +1717,11 @@
       <c r="E6" s="9" t="inlineStr"/>
       <c r="F6" s="9" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
@@ -1758,7 +1762,11 @@
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="9" t="inlineStr"/>
       <c r="G7" s="9" t="inlineStr"/>
-      <c r="H7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="9" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
@@ -1799,7 +1807,11 @@
       <c r="E8" s="9" t="inlineStr"/>
       <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="9" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
@@ -1840,7 +1852,11 @@
       <c r="E9" s="9" t="inlineStr"/>
       <c r="F9" s="9" t="inlineStr"/>
       <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="9" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="9" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
@@ -1881,7 +1897,11 @@
       <c r="E10" s="9" t="inlineStr"/>
       <c r="F10" s="9" t="inlineStr"/>
       <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="9" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="9" t="inlineStr"/>
       <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
@@ -1922,7 +1942,11 @@
       <c r="E11" s="9" t="inlineStr"/>
       <c r="F11" s="9" t="inlineStr"/>
       <c r="G11" s="9" t="inlineStr"/>
-      <c r="H11" s="9" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="9" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
@@ -1963,7 +1987,11 @@
       <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="9" t="inlineStr"/>
       <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="9" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="9" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
@@ -1998,7 +2026,11 @@
       <c r="E13" s="38" t="inlineStr"/>
       <c r="F13" s="38" t="inlineStr"/>
       <c r="G13" s="38" t="inlineStr"/>
-      <c r="H13" s="38" t="inlineStr"/>
+      <c r="H13" s="40" t="inlineStr">
+        <is>
+          <t>อินทัช เป็นสุข</t>
+        </is>
+      </c>
       <c r="I13" s="38" t="inlineStr"/>
       <c r="J13" s="38" t="inlineStr"/>
       <c r="K13" s="38" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for WELDING_ALUMINUM-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_WELDING_ALUMINUM-01.xlsx
+++ b/FM-MN-07_WELDING_ALUMINUM-01.xlsx
@@ -1722,7 +1722,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="9" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr"/>
@@ -1767,7 +1771,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="9" t="inlineStr"/>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr"/>
@@ -1812,7 +1820,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr"/>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
       <c r="L8" s="9" t="inlineStr"/>
@@ -1857,7 +1869,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr"/>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr"/>
@@ -1902,7 +1918,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="9" t="inlineStr"/>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr"/>
@@ -1947,7 +1967,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="9" t="inlineStr"/>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
@@ -1992,7 +2016,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="9" t="inlineStr"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr"/>
@@ -2031,7 +2059,11 @@
           <t>อินทัช เป็นสุข</t>
         </is>
       </c>
-      <c r="I13" s="38" t="inlineStr"/>
+      <c r="I13" s="40" t="inlineStr">
+        <is>
+          <t>อินทัช เป็นสุข</t>
+        </is>
+      </c>
       <c r="J13" s="38" t="inlineStr"/>
       <c r="K13" s="38" t="inlineStr"/>
       <c r="L13" s="38" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for WELDING_ALUMINUM-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_WELDING_ALUMINUM-01.xlsx
+++ b/FM-MN-07_WELDING_ALUMINUM-01.xlsx
@@ -1727,7 +1727,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="9" t="inlineStr"/>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="9" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr"/>
@@ -1776,7 +1780,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr"/>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="9" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr"/>
       <c r="M7" s="9" t="inlineStr"/>
@@ -1825,7 +1833,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr"/>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="9" t="inlineStr"/>
       <c r="L8" s="9" t="inlineStr"/>
       <c r="M8" s="9" t="inlineStr"/>
@@ -1874,7 +1886,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr"/>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="9" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr"/>
       <c r="M9" s="9" t="inlineStr"/>
@@ -1923,7 +1939,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="9" t="inlineStr"/>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr"/>
@@ -1972,7 +1992,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="9" t="inlineStr"/>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="9" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
       <c r="M11" s="9" t="inlineStr"/>
@@ -2021,7 +2045,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="9" t="inlineStr"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr"/>
@@ -2064,7 +2092,11 @@
           <t>อินทัช เป็นสุข</t>
         </is>
       </c>
-      <c r="J13" s="38" t="inlineStr"/>
+      <c r="J13" s="40" t="inlineStr">
+        <is>
+          <t>อินทัช เป็นสุข</t>
+        </is>
+      </c>
       <c r="K13" s="38" t="inlineStr"/>
       <c r="L13" s="38" t="inlineStr"/>
       <c r="M13" s="38" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for WELDING_ALUMINUM-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_WELDING_ALUMINUM-01.xlsx
+++ b/FM-MN-07_WELDING_ALUMINUM-01.xlsx
@@ -1733,7 +1733,11 @@
         </is>
       </c>
       <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="9" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="9" t="inlineStr"/>
       <c r="N6" s="9" t="inlineStr"/>
       <c r="O6" s="9" t="inlineStr"/>
@@ -1786,7 +1790,11 @@
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="9" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="9" t="inlineStr"/>
       <c r="N7" s="9" t="inlineStr"/>
       <c r="O7" s="9" t="inlineStr"/>
@@ -1839,7 +1847,11 @@
         </is>
       </c>
       <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="9" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="9" t="inlineStr"/>
       <c r="N8" s="9" t="inlineStr"/>
       <c r="O8" s="9" t="inlineStr"/>
@@ -1892,7 +1904,11 @@
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr"/>
-      <c r="L9" s="9" t="inlineStr"/>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="9" t="inlineStr"/>
       <c r="N9" s="9" t="inlineStr"/>
       <c r="O9" s="9" t="inlineStr"/>
@@ -1945,7 +1961,11 @@
         </is>
       </c>
       <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="9" t="inlineStr"/>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="9" t="inlineStr"/>
       <c r="N10" s="9" t="inlineStr"/>
       <c r="O10" s="9" t="inlineStr"/>
@@ -1998,7 +2018,11 @@
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="9" t="inlineStr"/>
+      <c r="L11" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="9" t="inlineStr"/>
       <c r="N11" s="9" t="inlineStr"/>
       <c r="O11" s="9" t="inlineStr"/>
@@ -2051,7 +2075,11 @@
         </is>
       </c>
       <c r="K12" s="9" t="inlineStr"/>
-      <c r="L12" s="9" t="inlineStr"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="9" t="inlineStr"/>
       <c r="N12" s="9" t="inlineStr"/>
       <c r="O12" s="9" t="inlineStr"/>
@@ -2098,7 +2126,11 @@
         </is>
       </c>
       <c r="K13" s="38" t="inlineStr"/>
-      <c r="L13" s="38" t="inlineStr"/>
+      <c r="L13" s="40" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="M13" s="38" t="inlineStr"/>
       <c r="N13" s="38" t="inlineStr"/>
       <c r="O13" s="38" t="inlineStr"/>

</xml_diff>